<commit_message>
Agregar documento de formalizacion para aval de RRHH
- Formalizacion-Proceso-Contable-RRHH.docx: descripcion de cargos con
  proposito, funciones, competencias y entregables por posicion; marco
  normativo con las nueve obligaciones de fecha legal; analisis de carga
  medida; matriz de riesgos de proceso y de continuidad; indicadores; y
  hoja de constancia con firmas de elaboracion, revision y aval.

- Informes-Gerencia-IES-2026.xlsx: se agrega portada con control
  documental y hoja de consolidado anual que enlaza con el seguimiento
  mensual. Verificadas las 60 formulas de la hoja 4 y los 12 enlaces
  cruzados del consolidado.

El esquema de reemplazos ante ausencias queda marcado como pendiente de
definicion, por requerir validacion de RRHH con las personas implicadas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VhbrSwAcj5Yomrrgr7yNVP
</commit_message>
<xml_diff>
--- a/ies-procesos/Informes-Gerencia-IES-2026.xlsx
+++ b/ies-procesos/Informes-Gerencia-IES-2026.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1 Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2 Ocupacion" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3 Calendario" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4 Gestion mensual" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="0 Portada" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1 Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2 Ocupacion" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3 Calendario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4 Gestion mensual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5 Consolidado" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,6 +128,23 @@
       <b val="1"/>
       <color rgb="00DC2626"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B3A6B"/>
+      <sz val="30"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A2540"/>
+      <sz val="17"/>
     </font>
   </fonts>
   <fills count="15">
@@ -271,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -396,6 +415,44 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -760,6 +817,272 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>IES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="50" t="inlineStr">
+        <is>
+          <t>Intelligent Electronic Solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>INFORME DE GESTIÓN DE PROCESOS CONTABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="50" t="inlineStr">
+        <is>
+          <t>Carga planificada, ocupación por posición y seguimiento mensual · 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="52" t="inlineStr">
+        <is>
+          <t>CONTROL DEL DOCUMENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="53" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>IES-CT-INF-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="53" t="inlineStr">
+        <is>
+          <t>Versión</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>Fecha de emisión</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>10 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="53" t="inlineStr">
+        <is>
+          <t>Elaborado por</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>Cristian Bernal — Contador</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="53" t="inlineStr">
+        <is>
+          <t>Dirigido a</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>Gerencia · Supervisión · Recursos Humanos</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="53" t="inlineStr">
+        <is>
+          <t>Periodicidad</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>Mensual, con corte al cierre de cada mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="53" t="inlineStr">
+        <is>
+          <t>Fuente de datos</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>Aplicación IES de seguimiento de procesos contables</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="53" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>Ciclo contable mensual — cinco posiciones del proceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="52" t="inlineStr">
+        <is>
+          <t>CONTENIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="55" t="inlineStr">
+        <is>
+          <t>1 Resumen</t>
+        </is>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>Carga anual por persona y concentración de la carga dentro del mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t>2 Ocupacion</t>
+        </is>
+      </c>
+      <c r="C22" s="54" t="inlineStr">
+        <is>
+          <t>Días-tarea de cada posición en los doce meses del año</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="55" t="inlineStr">
+        <is>
+          <t>3 Calendario</t>
+        </is>
+      </c>
+      <c r="C23" s="54" t="inlineStr">
+        <is>
+          <t>Hitos del ciclo con fecha límite y nivel de criticidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="55" t="inlineStr">
+        <is>
+          <t>4 Gestion mensual</t>
+        </is>
+      </c>
+      <c r="C24" s="54" t="inlineStr">
+        <is>
+          <t>Formato de seguimiento del cumplimiento real, mes a mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="55" t="inlineStr">
+        <is>
+          <t>5 Consolidado</t>
+        </is>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>Resumen anual del cumplimiento, se alimenta de la hoja 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>NOTA METODOLÓGICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="56" t="inlineStr">
+        <is>
+          <t>·  Días-tarea: suma de los días que cada tarea permanece abierta en el mes. Mide exposición y simultaneidad, no horas trabajadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="56" t="inlineStr">
+        <is>
+          <t>·  Ocupación: porcentaje de días del período con al menos una tarea abierta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="56" t="inlineStr">
+        <is>
+          <t>·  Pico: máximo de tareas de una misma persona abiertas en un mismo día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="56" t="inlineStr">
+        <is>
+          <t>·  Las hojas 1, 2 y 3 reflejan la carga PLANIFICADA según el catálogo de procesos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="56" t="inlineStr">
+        <is>
+          <t>·  La hoja 4 registra la EJECUCIÓN real y se diligencia al cierre de cada mes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B33:G33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
@@ -1132,8 +1455,8 @@
           <t>El 30% de la carga del mes cae entre los días 8 y 14. Coincide con el cierre contable y con los cinco insumos del informe.</t>
         </is>
       </c>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
+      <c r="D24" s="57" t="n"/>
+      <c r="E24" s="58" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="24" t="inlineStr">
@@ -1146,8 +1469,8 @@
           <t>15 tareas simultáneas del equipo el día 10, 12, 13. Es el punto más tenso del ciclo.</t>
         </is>
       </c>
-      <c r="D25" s="26" t="n"/>
-      <c r="E25" s="26" t="n"/>
+      <c r="D25" s="57" t="n"/>
+      <c r="E25" s="58" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="B26" s="24" t="inlineStr">
@@ -1160,8 +1483,8 @@
           <t>Pico de 7 tareas propias en un mismo día. Es la posición con la ventana más apretada del mes.</t>
         </is>
       </c>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="26" t="n"/>
+      <c r="D26" s="57" t="n"/>
+      <c r="E26" s="58" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="24" t="inlineStr">
@@ -1174,8 +1497,8 @@
           <t>Ocupación del 100%: tiene tareas abiertas todos los días del año por el registro diario de RC y RP.</t>
         </is>
       </c>
-      <c r="D27" s="26" t="n"/>
-      <c r="E27" s="26" t="n"/>
+      <c r="D27" s="57" t="n"/>
+      <c r="E27" s="58" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="24" t="inlineStr">
@@ -1188,8 +1511,8 @@
           <t>Dos compromisos con fecha: definir viáticos de tarjeta (días 6 a 10) y dar feedback al informe (días 13 a 14).</t>
         </is>
       </c>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
+      <c r="D28" s="57" t="n"/>
+      <c r="E28" s="58" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1204,7 +1527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1818,7 +2141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2394,7 +2717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2431,6 +2754,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -2459,6 +2783,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="35" t="inlineStr">
         <is>
@@ -2612,6 +2937,7 @@
       </c>
       <c r="G16" s="23" t="inlineStr"/>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="35" t="inlineStr">
         <is>
@@ -2765,6 +3091,7 @@
       </c>
       <c r="G25" s="23" t="inlineStr"/>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="B27" s="35" t="inlineStr">
         <is>
@@ -2918,6 +3245,7 @@
       </c>
       <c r="G34" s="23" t="inlineStr"/>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" s="35" t="inlineStr">
         <is>
@@ -3071,6 +3399,7 @@
       </c>
       <c r="G43" s="23" t="inlineStr"/>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="B45" s="35" t="inlineStr">
         <is>
@@ -3224,6 +3553,7 @@
       </c>
       <c r="G52" s="23" t="inlineStr"/>
     </row>
+    <row r="53"/>
     <row r="54">
       <c r="B54" s="35" t="inlineStr">
         <is>
@@ -3377,6 +3707,7 @@
       </c>
       <c r="G61" s="23" t="inlineStr"/>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="B63" s="35" t="inlineStr">
         <is>
@@ -3530,6 +3861,7 @@
       </c>
       <c r="G70" s="23" t="inlineStr"/>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="B72" s="35" t="inlineStr">
         <is>
@@ -3683,6 +4015,7 @@
       </c>
       <c r="G79" s="23" t="inlineStr"/>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="B81" s="35" t="inlineStr">
         <is>
@@ -3836,6 +4169,7 @@
       </c>
       <c r="G88" s="23" t="inlineStr"/>
     </row>
+    <row r="89"/>
     <row r="90">
       <c r="B90" s="35" t="inlineStr">
         <is>
@@ -3989,6 +4323,7 @@
       </c>
       <c r="G97" s="23" t="inlineStr"/>
     </row>
+    <row r="98"/>
     <row r="99">
       <c r="B99" s="35" t="inlineStr">
         <is>
@@ -4142,6 +4477,7 @@
       </c>
       <c r="G106" s="23" t="inlineStr"/>
     </row>
+    <row r="107"/>
     <row r="108">
       <c r="B108" s="35" t="inlineStr">
         <is>
@@ -4299,4 +4635,379 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>IES</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Consolidado anual de cumplimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Se alimenta automáticamente de la hoja 4 · no requiere diligenciamiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>Programadas</t>
+        </is>
+      </c>
+      <c r="D4" s="59" t="inlineStr">
+        <is>
+          <t>Completadas</t>
+        </is>
+      </c>
+      <c r="E4" s="59" t="inlineStr">
+        <is>
+          <t>Cumplimiento</t>
+        </is>
+      </c>
+      <c r="F4" s="59" t="inlineStr">
+        <is>
+          <t>Vencidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>Enero</t>
+        </is>
+      </c>
+      <c r="C5" s="60">
+        <f>'4 Gestion mensual'!C16</f>
+        <v/>
+      </c>
+      <c r="D5" s="60">
+        <f>'4 Gestion mensual'!D16</f>
+        <v/>
+      </c>
+      <c r="E5" s="61">
+        <f>IFERROR(D5/C5,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="60">
+        <f>'4 Gestion mensual'!F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>Febrero</t>
+        </is>
+      </c>
+      <c r="C6" s="60">
+        <f>'4 Gestion mensual'!C25</f>
+        <v/>
+      </c>
+      <c r="D6" s="60">
+        <f>'4 Gestion mensual'!D25</f>
+        <v/>
+      </c>
+      <c r="E6" s="61">
+        <f>IFERROR(D6/C6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="60">
+        <f>'4 Gestion mensual'!F25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="55" t="inlineStr">
+        <is>
+          <t>Marzo</t>
+        </is>
+      </c>
+      <c r="C7" s="60">
+        <f>'4 Gestion mensual'!C34</f>
+        <v/>
+      </c>
+      <c r="D7" s="60">
+        <f>'4 Gestion mensual'!D34</f>
+        <v/>
+      </c>
+      <c r="E7" s="61">
+        <f>IFERROR(D7/C7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="60">
+        <f>'4 Gestion mensual'!F34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="C8" s="60">
+        <f>'4 Gestion mensual'!C43</f>
+        <v/>
+      </c>
+      <c r="D8" s="60">
+        <f>'4 Gestion mensual'!D43</f>
+        <v/>
+      </c>
+      <c r="E8" s="61">
+        <f>IFERROR(D8/C8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="60">
+        <f>'4 Gestion mensual'!F43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="55" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C9" s="60">
+        <f>'4 Gestion mensual'!C52</f>
+        <v/>
+      </c>
+      <c r="D9" s="60">
+        <f>'4 Gestion mensual'!D52</f>
+        <v/>
+      </c>
+      <c r="E9" s="61">
+        <f>IFERROR(D9/C9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="60">
+        <f>'4 Gestion mensual'!F52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C10" s="60">
+        <f>'4 Gestion mensual'!C61</f>
+        <v/>
+      </c>
+      <c r="D10" s="60">
+        <f>'4 Gestion mensual'!D61</f>
+        <v/>
+      </c>
+      <c r="E10" s="61">
+        <f>IFERROR(D10/C10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="60">
+        <f>'4 Gestion mensual'!F61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="55" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C11" s="60">
+        <f>'4 Gestion mensual'!C70</f>
+        <v/>
+      </c>
+      <c r="D11" s="60">
+        <f>'4 Gestion mensual'!D70</f>
+        <v/>
+      </c>
+      <c r="E11" s="61">
+        <f>IFERROR(D11/C11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="60">
+        <f>'4 Gestion mensual'!F70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="55" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="C12" s="60">
+        <f>'4 Gestion mensual'!C79</f>
+        <v/>
+      </c>
+      <c r="D12" s="60">
+        <f>'4 Gestion mensual'!D79</f>
+        <v/>
+      </c>
+      <c r="E12" s="61">
+        <f>IFERROR(D12/C12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="60">
+        <f>'4 Gestion mensual'!F79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Septiembre</t>
+        </is>
+      </c>
+      <c r="C13" s="60">
+        <f>'4 Gestion mensual'!C88</f>
+        <v/>
+      </c>
+      <c r="D13" s="60">
+        <f>'4 Gestion mensual'!D88</f>
+        <v/>
+      </c>
+      <c r="E13" s="61">
+        <f>IFERROR(D13/C13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="60">
+        <f>'4 Gestion mensual'!F88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="55" t="inlineStr">
+        <is>
+          <t>Octubre</t>
+        </is>
+      </c>
+      <c r="C14" s="60">
+        <f>'4 Gestion mensual'!C97</f>
+        <v/>
+      </c>
+      <c r="D14" s="60">
+        <f>'4 Gestion mensual'!D97</f>
+        <v/>
+      </c>
+      <c r="E14" s="61">
+        <f>IFERROR(D14/C14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="60">
+        <f>'4 Gestion mensual'!F97</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="55" t="inlineStr">
+        <is>
+          <t>Noviembre</t>
+        </is>
+      </c>
+      <c r="C15" s="60">
+        <f>'4 Gestion mensual'!C106</f>
+        <v/>
+      </c>
+      <c r="D15" s="60">
+        <f>'4 Gestion mensual'!D106</f>
+        <v/>
+      </c>
+      <c r="E15" s="61">
+        <f>IFERROR(D15/C15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="60">
+        <f>'4 Gestion mensual'!F106</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="55" t="inlineStr">
+        <is>
+          <t>Diciembre</t>
+        </is>
+      </c>
+      <c r="C16" s="60">
+        <f>'4 Gestion mensual'!C115</f>
+        <v/>
+      </c>
+      <c r="D16" s="60">
+        <f>'4 Gestion mensual'!D115</f>
+        <v/>
+      </c>
+      <c r="E16" s="61">
+        <f>IFERROR(D16/C16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="60">
+        <f>'4 Gestion mensual'!F115</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="53" t="inlineStr">
+        <is>
+          <t>TOTAL AÑO</t>
+        </is>
+      </c>
+      <c r="C17" s="62">
+        <f>SUM(C5:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="62">
+        <f>SUM(D5:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="63">
+        <f>IFERROR(D17/C17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="62">
+        <f>SUM(F5:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="64" t="inlineStr">
+        <is>
+          <t>Las celdas de esta hoja se calculan solas. Para que muestren datos, diligencie primero la hoja 4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
 </file>
</xml_diff>